<commit_message>
chore: update northbound mutual fund AUM
</commit_message>
<xml_diff>
--- a/outputs/latest.xlsx
+++ b/outputs/latest.xlsx
@@ -247,7 +247,7 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: Link discovery failed for https://www.schroders.com/en-hk/hk/individual: HTTPSConnectionPool(host='www.schroders.com', port=443): Read timed out. (read timeout=15) | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K14" authorId="0" shapeId="0">
@@ -268,7 +268,7 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K17" authorId="0" shapeId="0">
@@ -349,7 +349,7 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K28" authorId="0" shapeId="0">
@@ -567,7 +567,7 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: Link discovery failed for https://www.schroders.com/en-hk/hk/individual: HTTPSConnectionPool(host='www.schroders.com', port=443): Read timed out. (read timeout=15) | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K14" authorId="0" shapeId="0">
@@ -707,28 +707,28 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K34" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K35" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K36" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K37" authorId="0" shapeId="0">
@@ -875,35 +875,35 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K58" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K59" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K60" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K61" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K62" authorId="0" shapeId="0">
@@ -1389,21 +1389,21 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: Link discovery failed for https://www.schroders.com/en-hk/hk/individual: HTTPSConnectionPool(host='www.schroders.com', port=443): Read timed out. (read timeout=15) | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K132" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: Link discovery failed for https://www.schroders.com/en-hk/hk/individual: HTTPSConnectionPool(host='www.schroders.com', port=443): Read timed out. (read timeout=15) | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K133" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 施罗德投资管理(香港)
-抓取信息: Link discovery failed for https://www.schroders.com/en-hk/hk/individual: HTTPSConnectionPool(host='www.schroders.com', port=443): Read timed out. (read timeout=15) | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
+抓取信息: No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K134" authorId="0" shapeId="0">
@@ -2118,98 +2118,98 @@
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K237" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K238" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K239" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K240" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K241" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K242" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K243" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K244" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K245" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K246" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K247" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K248" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
     <comment ref="K249" authorId="0" shapeId="0">
       <text>
         <t>未抓到最新规模，单元格留空。
 基金管理人: 惠理基金(香港)
-抓取信息: Fetch failed for https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/ftp/files/reports/hdlv/001_fact_sheet/eng/hdlv_fact_sheet_2026-01-01_en.pdf | Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted.</t>
+抓取信息: Fetch failed for https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf: 404 Client Error: Not Found for url: https://www.valuepartners-group.com/doc/notice/20170421_Notice_to_Investors_VP_Funds_Ongoing_Charges_E.pdf | No global fund AUM evidence extracted. | No mainland share-class AUM evidence extracted.</t>
       </text>
     </comment>
   </commentList>
@@ -2584,7 +2584,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>最新基金规模合计(亿人民币）（2026-08-17）</t>
+          <t>最新基金规模合计(亿人民币）（2026-08-24）</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -3388,7 +3388,7 @@
         <v>205.1814078</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>165.01955</v>
+        <v>164.509409</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -3481,7 +3481,7 @@
         <v>56.13075468</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>51.408925</v>
+        <v>51.25</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -4280,7 +4280,7 @@
         <v>211.61545812</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>207.455845</v>
+        <v>206.814516</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
         <v>256.38451344</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>166.421734</v>
+        <v>165.907258</v>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
@@ -4557,7 +4557,7 @@
         <v>72.6859386</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>129.223406</v>
+        <v>128.823925</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
         <v>46.77112908</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>57.287313</v>
+        <v>57.110215</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
@@ -6659,7 +6659,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>最新基金规模合计(亿人民币）（2026-08-17）</t>
+          <t>最新基金规模合计(亿人民币）（2026-08-24）</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">

</xml_diff>